<commit_message>
Remove Module 0 from extraction tracker
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/extraction-tracker.xlsx
+++ b/extraction-tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Extraction Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Extraction Tracker'!$A$1:$H$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Extraction Tracker'!$A$1:$H$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -523,7 +523,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
@@ -547,7 +547,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B3" s="5" t="n">
@@ -571,7 +571,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
@@ -595,7 +595,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
@@ -619,7 +619,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
@@ -639,7 +639,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
@@ -659,7 +659,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
@@ -679,7 +679,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -699,7 +699,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
@@ -719,7 +719,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -739,7 +739,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
@@ -759,7 +759,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
@@ -779,7 +779,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
@@ -799,7 +799,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
@@ -819,7 +819,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
@@ -839,7 +839,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
@@ -859,7 +859,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
@@ -879,7 +879,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
@@ -899,7 +899,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
@@ -919,7 +919,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Module 0</t>
+          <t>Module 1</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
@@ -939,7 +939,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
@@ -948,11 +948,7 @@
       <c r="C22" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Fraction Gymnastics</t>
-        </is>
-      </c>
+      <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="n">
         <v>8</v>
       </c>
@@ -963,7 +959,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
@@ -972,11 +968,7 @@
       <c r="C23" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Continued Fraction</t>
-        </is>
-      </c>
+      <c r="D23" s="4" t="inlineStr"/>
       <c r="E23" s="5" t="n">
         <v>8</v>
       </c>
@@ -987,7 +979,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
@@ -996,11 +988,7 @@
       <c r="C24" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Comparing Fractions</t>
-        </is>
-      </c>
+      <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="3" t="n">
         <v>8</v>
       </c>
@@ -1011,7 +999,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
@@ -1020,11 +1008,7 @@
       <c r="C25" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Sports</t>
-        </is>
-      </c>
+      <c r="D25" s="4" t="inlineStr"/>
       <c r="E25" s="5" t="n">
         <v>8</v>
       </c>
@@ -1035,7 +1019,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B26" s="3" t="n">
@@ -1055,7 +1039,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
@@ -1075,7 +1059,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
@@ -1095,7 +1079,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
@@ -1115,7 +1099,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
@@ -1135,7 +1119,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
@@ -1155,7 +1139,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B32" s="3" t="n">
@@ -1175,7 +1159,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
@@ -1195,7 +1179,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
@@ -1215,7 +1199,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B35" s="5" t="n">
@@ -1235,7 +1219,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
@@ -1255,7 +1239,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B37" s="5" t="n">
@@ -1275,7 +1259,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
@@ -1295,7 +1279,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B39" s="5" t="n">
@@ -1315,7 +1299,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
@@ -1335,7 +1319,7 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Module 1</t>
+          <t>Module 2</t>
         </is>
       </c>
       <c r="B41" s="5" t="n">
@@ -1355,7 +1339,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B42" s="3" t="n">
@@ -1375,7 +1359,7 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
@@ -1395,7 +1379,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
@@ -1415,7 +1399,7 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
@@ -1435,7 +1419,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B46" s="3" t="n">
@@ -1455,7 +1439,7 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
@@ -1475,7 +1459,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B48" s="3" t="n">
@@ -1495,7 +1479,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B49" s="5" t="n">
@@ -1515,7 +1499,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
@@ -1535,7 +1519,7 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B51" s="5" t="n">
@@ -1555,7 +1539,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B52" s="3" t="n">
@@ -1575,7 +1559,7 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B53" s="5" t="n">
@@ -1595,7 +1579,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B54" s="3" t="n">
@@ -1615,7 +1599,7 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B55" s="5" t="n">
@@ -1635,7 +1619,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B56" s="3" t="n">
@@ -1655,7 +1639,7 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B57" s="5" t="n">
@@ -1675,7 +1659,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B58" s="3" t="n">
@@ -1695,7 +1679,7 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B59" s="5" t="n">
@@ -1715,7 +1699,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B60" s="3" t="n">
@@ -1735,7 +1719,7 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>Module 2</t>
+          <t>Module 3</t>
         </is>
       </c>
       <c r="B61" s="5" t="n">
@@ -1755,7 +1739,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B62" s="3" t="n">
@@ -1775,7 +1759,7 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B63" s="5" t="n">
@@ -1795,7 +1779,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B64" s="3" t="n">
@@ -1815,7 +1799,7 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B65" s="5" t="n">
@@ -1835,7 +1819,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B66" s="3" t="n">
@@ -1855,7 +1839,7 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B67" s="5" t="n">
@@ -1875,7 +1859,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B68" s="3" t="n">
@@ -1895,7 +1879,7 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B69" s="5" t="n">
@@ -1915,7 +1899,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B70" s="3" t="n">
@@ -1935,7 +1919,7 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B71" s="5" t="n">
@@ -1955,7 +1939,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B72" s="3" t="n">
@@ -1975,7 +1959,7 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B73" s="5" t="n">
@@ -1995,7 +1979,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B74" s="3" t="n">
@@ -2015,7 +1999,7 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B75" s="5" t="n">
@@ -2035,7 +2019,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B76" s="3" t="n">
@@ -2055,7 +2039,7 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B77" s="5" t="n">
@@ -2075,7 +2059,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B78" s="3" t="n">
@@ -2095,7 +2079,7 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B79" s="5" t="n">
@@ -2115,7 +2099,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B80" s="3" t="n">
@@ -2135,7 +2119,7 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>Module 3</t>
+          <t>Workout 1A</t>
         </is>
       </c>
       <c r="B81" s="5" t="n">
@@ -2155,7 +2139,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B82" s="3" t="n">
@@ -2175,7 +2159,7 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B83" s="5" t="n">
@@ -2195,7 +2179,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B84" s="3" t="n">
@@ -2215,7 +2199,7 @@
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B85" s="5" t="n">
@@ -2235,7 +2219,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B86" s="3" t="n">
@@ -2255,7 +2239,7 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B87" s="5" t="n">
@@ -2275,7 +2259,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B88" s="3" t="n">
@@ -2295,7 +2279,7 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B89" s="5" t="n">
@@ -2315,7 +2299,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B90" s="3" t="n">
@@ -2335,7 +2319,7 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B91" s="5" t="n">
@@ -2355,7 +2339,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B92" s="3" t="n">
@@ -2375,7 +2359,7 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B93" s="5" t="n">
@@ -2395,7 +2379,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B94" s="3" t="n">
@@ -2415,7 +2399,7 @@
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B95" s="5" t="n">
@@ -2435,7 +2419,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B96" s="3" t="n">
@@ -2455,7 +2439,7 @@
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B97" s="5" t="n">
@@ -2475,7 +2459,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B98" s="3" t="n">
@@ -2495,7 +2479,7 @@
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B99" s="5" t="n">
@@ -2515,7 +2499,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B100" s="3" t="n">
@@ -2535,7 +2519,7 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>Workout 1A</t>
+          <t>Workout 1B</t>
         </is>
       </c>
       <c r="B101" s="5" t="n">
@@ -2552,408 +2536,8 @@
       <c r="G101" s="4" t="inlineStr"/>
       <c r="H101" s="4" t="inlineStr"/>
     </row>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B102" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C102" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D102" s="2" t="inlineStr"/>
-      <c r="E102" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F102" s="2" t="inlineStr"/>
-      <c r="G102" s="2" t="inlineStr"/>
-      <c r="H102" s="2" t="inlineStr"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="4" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B103" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C103" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D103" s="4" t="inlineStr"/>
-      <c r="E103" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F103" s="4" t="inlineStr"/>
-      <c r="G103" s="4" t="inlineStr"/>
-      <c r="H103" s="4" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B104" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C104" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D104" s="2" t="inlineStr"/>
-      <c r="E104" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F104" s="2" t="inlineStr"/>
-      <c r="G104" s="2" t="inlineStr"/>
-      <c r="H104" s="2" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="4" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B105" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C105" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="D105" s="4" t="inlineStr"/>
-      <c r="E105" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F105" s="4" t="inlineStr"/>
-      <c r="G105" s="4" t="inlineStr"/>
-      <c r="H105" s="4" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B106" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C106" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D106" s="2" t="inlineStr"/>
-      <c r="E106" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F106" s="2" t="inlineStr"/>
-      <c r="G106" s="2" t="inlineStr"/>
-      <c r="H106" s="2" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="4" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B107" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C107" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D107" s="4" t="inlineStr"/>
-      <c r="E107" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F107" s="4" t="inlineStr"/>
-      <c r="G107" s="4" t="inlineStr"/>
-      <c r="H107" s="4" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B108" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C108" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D108" s="2" t="inlineStr"/>
-      <c r="E108" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F108" s="2" t="inlineStr"/>
-      <c r="G108" s="2" t="inlineStr"/>
-      <c r="H108" s="2" t="inlineStr"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="4" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B109" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C109" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D109" s="4" t="inlineStr"/>
-      <c r="E109" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F109" s="4" t="inlineStr"/>
-      <c r="G109" s="4" t="inlineStr"/>
-      <c r="H109" s="4" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B110" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C110" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D110" s="2" t="inlineStr"/>
-      <c r="E110" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F110" s="2" t="inlineStr"/>
-      <c r="G110" s="2" t="inlineStr"/>
-      <c r="H110" s="2" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="4" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B111" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C111" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="D111" s="4" t="inlineStr"/>
-      <c r="E111" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F111" s="4" t="inlineStr"/>
-      <c r="G111" s="4" t="inlineStr"/>
-      <c r="H111" s="4" t="inlineStr"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B112" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C112" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D112" s="2" t="inlineStr"/>
-      <c r="E112" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F112" s="2" t="inlineStr"/>
-      <c r="G112" s="2" t="inlineStr"/>
-      <c r="H112" s="2" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="4" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B113" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C113" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D113" s="4" t="inlineStr"/>
-      <c r="E113" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F113" s="4" t="inlineStr"/>
-      <c r="G113" s="4" t="inlineStr"/>
-      <c r="H113" s="4" t="inlineStr"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B114" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C114" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D114" s="2" t="inlineStr"/>
-      <c r="E114" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F114" s="2" t="inlineStr"/>
-      <c r="G114" s="2" t="inlineStr"/>
-      <c r="H114" s="2" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="4" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B115" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C115" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="D115" s="4" t="inlineStr"/>
-      <c r="E115" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F115" s="4" t="inlineStr"/>
-      <c r="G115" s="4" t="inlineStr"/>
-      <c r="H115" s="4" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B116" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C116" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D116" s="2" t="inlineStr"/>
-      <c r="E116" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F116" s="2" t="inlineStr"/>
-      <c r="G116" s="2" t="inlineStr"/>
-      <c r="H116" s="2" t="inlineStr"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="4" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B117" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C117" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D117" s="4" t="inlineStr"/>
-      <c r="E117" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F117" s="4" t="inlineStr"/>
-      <c r="G117" s="4" t="inlineStr"/>
-      <c r="H117" s="4" t="inlineStr"/>
-    </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B118" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="C118" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D118" s="2" t="inlineStr"/>
-      <c r="E118" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F118" s="2" t="inlineStr"/>
-      <c r="G118" s="2" t="inlineStr"/>
-      <c r="H118" s="2" t="inlineStr"/>
-    </row>
-    <row r="119">
-      <c r="A119" s="4" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B119" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C119" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D119" s="4" t="inlineStr"/>
-      <c r="E119" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F119" s="4" t="inlineStr"/>
-      <c r="G119" s="4" t="inlineStr"/>
-      <c r="H119" s="4" t="inlineStr"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="2" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B120" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="C120" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D120" s="2" t="inlineStr"/>
-      <c r="E120" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F120" s="2" t="inlineStr"/>
-      <c r="G120" s="2" t="inlineStr"/>
-      <c r="H120" s="2" t="inlineStr"/>
-    </row>
-    <row r="121">
-      <c r="A121" s="4" t="inlineStr">
-        <is>
-          <t>Workout 1B</t>
-        </is>
-      </c>
-      <c r="B121" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C121" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="D121" s="4" t="inlineStr"/>
-      <c r="E121" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F121" s="4" t="inlineStr"/>
-      <c r="G121" s="4" t="inlineStr"/>
-      <c r="H121" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H121"/>
+  <autoFilter ref="A1:H101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>